<commit_message>
fix(build): resolve typescript definitions for production render deployment and update levels sheet
</commit_message>
<xml_diff>
--- a/Assessment_4_Sudharshanan.xlsx
+++ b/Assessment_4_Sudharshanan.xlsx
@@ -1335,7 +1335,11 @@
           <t>2_Must_haves ; tests/**/*.test.ts (55/55 tests passing)</t>
         </is>
       </c>
-      <c r="E5" s="7" t="n"/>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Command: npm test (55/55 passed) | URL: http://localhost:3000 | Files: tests/**/*.test.ts, REPORT.md Sec 2, TEST_INDEX.md</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1358,7 +1362,11 @@
           <t>data/certification/*_evidence.json ; npm run test:certification</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Command: npm run test:certification | URL: http://localhost:2368/about/ | Files: data/certification/*_evidence.json, src/certification/runner.ts</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1381,7 +1389,11 @@
           <t>src/connectors/base.ts ; src/manifests/*.yaml (error_map)</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n"/>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Command: npx jest tests/contract/connectors.test.ts | Files: src/connectors/base.ts (mapError), src/manifests/*.yaml, src/middleware/errorHandler.ts</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="69.75" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1404,7 +1416,11 @@
           <t>src/catalogue/importer.ts ; tests/unit/advanced.test.ts (1,000 rows in 21ms)</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n"/>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Command: npx jest tests/unit/advanced.test.ts -t "Catalogue CSV Import" (1,000 rows in 21ms) | URL: POST /api/v1/catalogue/import | Files: src/catalogue/importer.ts</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1427,7 +1443,11 @@
           <t>src/rules/ai_capture.ts ; tests/unit/advanced.test.ts</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Command: npx jest tests/unit/advanced.test.ts -t "AI Rules Capture" | URL: POST /api/v1/rules/propose &amp; POST /api/v1/rules/confirm | Files: src/rules/capture.ts</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="27.75" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -1450,7 +1470,11 @@
           <t>src/rules/relevance.ts ; tests/unit/advanced.test.ts</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Command: npx jest tests/unit/advanced.test.ts -t "Audience Relevance Scorer" | URL: GET /api/v1/destinations | Files: src/catalogue/store.ts, src/catalogue/tailoring.ts</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="55.5" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -1473,7 +1497,11 @@
           <t>src/tailoring/engine.ts ; tests/unit/advanced.test.ts</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n"/>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Command: npx jest tests/unit/advanced.test.ts -t "Content Tailoring Engine" | URL: POST /api/v1/tailor | Files: src/catalogue/tailoring.ts</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -1496,7 +1524,11 @@
           <t>src/connectors/hashnode.ts ; src/connectors/slack.ts ; src/connectors/mrss.ts</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n"/>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Command: npm run test:certification (verifies Hashnode, Slack, MRSS) | URL: GET /connector/v1/{hashnode,slack,mrss}/manifest | Files: src/connectors/{hashnode,slack,mrss}.ts</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -1519,7 +1551,11 @@
           <t>Skipped per 4-day prioritized battle plan</t>
         </is>
       </c>
-      <c r="E13" s="7" t="n"/>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Skipped per 4-day prioritized battle plan | Documented in REPORT.md Section 5</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="27.75" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -1542,7 +1578,11 @@
           <t>fetch_metrics implemented on Dev.to, Discourse, Lemmy, Ghost, and Hashnode</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Command: npx tsx -e "import { globalRegistry } from './src/connectors/registry.js'; (async () =&gt; console.log(await globalRegistry.get('ghost').fetchMetrics('1', {})))()" | Files: src/connectors/ghost.ts, devto.ts, lemmy.ts</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -1565,7 +1605,11 @@
           <t>Skipped per 4-day prioritized battle plan</t>
         </is>
       </c>
-      <c r="E15" s="7" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Skipped per 4-day prioritized battle plan | Documented in REPORT.md Section 5</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -1588,7 +1632,11 @@
           <t>Skipped per 4-day prioritized battle plan</t>
         </is>
       </c>
-      <c r="E16" s="7" t="n"/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Skipped per 4-day prioritized battle plan | Documented in REPORT.md Section 5</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="3" t="inlineStr">

</xml_diff>